<commit_message>
panchapale 2 estimates for bhimsen mandir complete
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/thekka/कृषि उपज संकलन केन्द्र निर्माण - शंखरापुर -१/कृषि उपज संकलन केन्द्र निर्माण - शंखरापुर -१.xlsx
+++ b/बजेट माग estimate/thekka/कृषि उपज संकलन केन्द्र निर्माण - शंखरापुर -१/कृषि उपज संकलन केन्द्र निर्माण - शंखरापुर -१.xlsx
@@ -1,11 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D5618C2-409A-4CC4-B70D-27F9F5D3E684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="estimate" sheetId="13" r:id="rId1"/>
@@ -34,11 +33,11 @@
     <definedName name="description_783">[1]Abstract!$B$301</definedName>
     <definedName name="description_784">[3]Abstract!$B$300</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">estimate!$A$1:$K$158</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">krishi!$A$1:$K$97</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">krishi!$A$1:$K$101</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">estimate!$1:$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">krishi!$1:$8</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -56,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="126">
   <si>
     <t>Government of Nepal</t>
   </si>
@@ -650,14 +649,17 @@
       <t xml:space="preserve"> s[lif pkh ;+sng s]Gb| lgdf{0f</t>
     </r>
   </si>
+  <si>
+    <t>l;d]G6 jf jh|df hf]8]sf] uf/f] eTsfO{ To;af6 cfPsf] ;fdfu+|L !) dL</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="17" x14ac:knownFonts="1">
     <font>
@@ -828,9 +830,9 @@
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
@@ -846,14 +848,14 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="43" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -882,7 +884,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -919,7 +921,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -937,7 +939,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -946,46 +948,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1008,14 +973,51 @@
     <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Comma 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Comma 2" xfId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
-    <cellStyle name="Normal 3" xfId="5" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
-    <cellStyle name="Percent 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
+    <cellStyle name="Normal 2" xfId="2"/>
+    <cellStyle name="Normal 3" xfId="5"/>
+    <cellStyle name="Percent 2" xfId="4"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -1031,7 +1033,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -1125,7 +1127,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -1184,7 +1186,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -1248,9 +1250,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1288,9 +1290,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1325,7 +1327,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1360,7 +1362,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1533,7 +1535,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:M158"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1549,113 +1551,113 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
-      <c r="I1" s="49"/>
-      <c r="J1" s="49"/>
-      <c r="K1" s="49"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
     </row>
     <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
-      <c r="E2" s="50"/>
-      <c r="F2" s="50"/>
-      <c r="G2" s="50"/>
-      <c r="H2" s="50"/>
-      <c r="I2" s="50"/>
-      <c r="J2" s="50"/>
-      <c r="K2" s="50"/>
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="62"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="51" t="s">
+      <c r="A3" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="51"/>
-      <c r="C3" s="51"/>
-      <c r="D3" s="51"/>
-      <c r="E3" s="51"/>
-      <c r="F3" s="51"/>
-      <c r="G3" s="51"/>
-      <c r="H3" s="51"/>
-      <c r="I3" s="51"/>
-      <c r="J3" s="51"/>
-      <c r="K3" s="51"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
+      <c r="K3" s="63"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="51" t="s">
+      <c r="A4" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="51"/>
-      <c r="C4" s="51"/>
-      <c r="D4" s="51"/>
-      <c r="E4" s="51"/>
-      <c r="F4" s="51"/>
-      <c r="G4" s="51"/>
-      <c r="H4" s="51"/>
-      <c r="I4" s="51"/>
-      <c r="J4" s="51"/>
-      <c r="K4" s="51"/>
+      <c r="B4" s="63"/>
+      <c r="C4" s="63"/>
+      <c r="D4" s="63"/>
+      <c r="E4" s="63"/>
+      <c r="F4" s="63"/>
+      <c r="G4" s="63"/>
+      <c r="H4" s="63"/>
+      <c r="I4" s="63"/>
+      <c r="J4" s="63"/>
+      <c r="K4" s="63"/>
     </row>
     <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="52" t="s">
+      <c r="A5" s="64" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="52"/>
-      <c r="C5" s="52"/>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
-      <c r="G5" s="52"/>
-      <c r="H5" s="52"/>
-      <c r="I5" s="52"/>
-      <c r="J5" s="52"/>
-      <c r="K5" s="52"/>
+      <c r="B5" s="64"/>
+      <c r="C5" s="64"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
+      <c r="I5" s="64"/>
+      <c r="J5" s="64"/>
+      <c r="K5" s="64"/>
     </row>
     <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="47" t="s">
+      <c r="A6" s="65" t="s">
         <v>86</v>
       </c>
-      <c r="B6" s="47"/>
-      <c r="C6" s="47"/>
-      <c r="D6" s="47"/>
-      <c r="E6" s="47"/>
-      <c r="F6" s="47"/>
+      <c r="B6" s="65"/>
+      <c r="C6" s="65"/>
+      <c r="D6" s="65"/>
+      <c r="E6" s="65"/>
+      <c r="F6" s="65"/>
       <c r="G6" s="4"/>
-      <c r="H6" s="48" t="s">
+      <c r="H6" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="I6" s="48"/>
-      <c r="J6" s="48"/>
-      <c r="K6" s="48"/>
+      <c r="I6" s="66"/>
+      <c r="J6" s="66"/>
+      <c r="K6" s="66"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="55" t="s">
+      <c r="A7" s="59" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="55"/>
-      <c r="C7" s="55"/>
-      <c r="D7" s="55"/>
-      <c r="E7" s="55"/>
-      <c r="F7" s="55"/>
+      <c r="B7" s="59"/>
+      <c r="C7" s="59"/>
+      <c r="D7" s="59"/>
+      <c r="E7" s="59"/>
+      <c r="F7" s="59"/>
       <c r="G7" s="5"/>
-      <c r="H7" s="56" t="s">
+      <c r="H7" s="60" t="s">
         <v>88</v>
       </c>
-      <c r="I7" s="56"/>
-      <c r="J7" s="56"/>
-      <c r="K7" s="56"/>
+      <c r="I7" s="60"/>
+      <c r="J7" s="60"/>
+      <c r="K7" s="60"/>
     </row>
     <row r="8" spans="1:11" s="10" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
@@ -4958,11 +4960,11 @@
       <c r="B153" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="C153" s="53">
+      <c r="C153" s="54">
         <f>J151</f>
         <v>520268.58119831659</v>
       </c>
-      <c r="D153" s="54"/>
+      <c r="D153" s="55"/>
       <c r="E153" s="39">
         <v>100</v>
       </c>
@@ -4977,21 +4979,21 @@
       <c r="B154" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="C154" s="57">
+      <c r="C154" s="56">
         <v>700000</v>
       </c>
-      <c r="D154" s="58"/>
+      <c r="D154" s="57"/>
       <c r="E154" s="39"/>
     </row>
     <row r="155" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B155" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="C155" s="57">
+      <c r="C155" s="56">
         <f>C154-C157-C158</f>
         <v>665000</v>
       </c>
-      <c r="D155" s="58"/>
+      <c r="D155" s="57"/>
       <c r="E155" s="39">
         <f>C155/C153*100</f>
         <v>127.81859678482381</v>
@@ -5001,11 +5003,11 @@
       <c r="B156" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="C156" s="59">
+      <c r="C156" s="58">
         <f>C153-C155</f>
         <v>-144731.41880168341</v>
       </c>
-      <c r="D156" s="59"/>
+      <c r="D156" s="58"/>
       <c r="E156" s="39">
         <f>100-E155</f>
         <v>-27.818596784823811</v>
@@ -5015,11 +5017,11 @@
       <c r="B157" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="C157" s="53">
+      <c r="C157" s="54">
         <f>C154*0.03</f>
         <v>21000</v>
       </c>
-      <c r="D157" s="54"/>
+      <c r="D157" s="55"/>
       <c r="E157" s="39">
         <v>3</v>
       </c>
@@ -5028,23 +5030,17 @@
       <c r="B158" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="C158" s="53">
+      <c r="C158" s="54">
         <f>C154*0.02</f>
         <v>14000</v>
       </c>
-      <c r="D158" s="54"/>
+      <c r="D158" s="55"/>
       <c r="E158" s="39">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="C158:D158"/>
-    <mergeCell ref="C153:D153"/>
-    <mergeCell ref="C154:D154"/>
-    <mergeCell ref="C155:D155"/>
-    <mergeCell ref="C156:D156"/>
-    <mergeCell ref="C157:D157"/>
     <mergeCell ref="A7:F7"/>
     <mergeCell ref="H7:K7"/>
     <mergeCell ref="A1:K1"/>
@@ -5054,6 +5050,12 @@
     <mergeCell ref="A5:K5"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="H6:K6"/>
+    <mergeCell ref="C158:D158"/>
+    <mergeCell ref="C153:D153"/>
+    <mergeCell ref="C154:D154"/>
+    <mergeCell ref="C155:D155"/>
+    <mergeCell ref="C156:D156"/>
+    <mergeCell ref="C157:D157"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="80" orientation="portrait" r:id="rId1"/>
@@ -5064,8 +5066,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K97"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K101"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.7109375" style="14" customWidth="1"/>
@@ -5080,116 +5082,116 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
-      <c r="I1" s="49"/>
-      <c r="J1" s="49"/>
-      <c r="K1" s="49"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
     </row>
     <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="62" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
-      <c r="E2" s="50"/>
-      <c r="F2" s="50"/>
-      <c r="G2" s="50"/>
-      <c r="H2" s="50"/>
-      <c r="I2" s="50"/>
-      <c r="J2" s="50"/>
-      <c r="K2" s="50"/>
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="62"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="51" t="s">
+      <c r="A3" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="51"/>
-      <c r="C3" s="51"/>
-      <c r="D3" s="51"/>
-      <c r="E3" s="51"/>
-      <c r="F3" s="51"/>
-      <c r="G3" s="51"/>
-      <c r="H3" s="51"/>
-      <c r="I3" s="51"/>
-      <c r="J3" s="51"/>
-      <c r="K3" s="51"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
+      <c r="K3" s="63"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="51" t="s">
+      <c r="A4" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="51"/>
-      <c r="C4" s="51"/>
-      <c r="D4" s="51"/>
-      <c r="E4" s="51"/>
-      <c r="F4" s="51"/>
-      <c r="G4" s="51"/>
-      <c r="H4" s="51"/>
-      <c r="I4" s="51"/>
-      <c r="J4" s="51"/>
-      <c r="K4" s="51"/>
+      <c r="B4" s="63"/>
+      <c r="C4" s="63"/>
+      <c r="D4" s="63"/>
+      <c r="E4" s="63"/>
+      <c r="F4" s="63"/>
+      <c r="G4" s="63"/>
+      <c r="H4" s="63"/>
+      <c r="I4" s="63"/>
+      <c r="J4" s="63"/>
+      <c r="K4" s="63"/>
     </row>
     <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="52" t="s">
+      <c r="A5" s="64" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="52"/>
-      <c r="C5" s="52"/>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
-      <c r="G5" s="52"/>
-      <c r="H5" s="52"/>
-      <c r="I5" s="52"/>
-      <c r="J5" s="52"/>
-      <c r="K5" s="52"/>
+      <c r="B5" s="64"/>
+      <c r="C5" s="64"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
+      <c r="I5" s="64"/>
+      <c r="J5" s="64"/>
+      <c r="K5" s="64"/>
     </row>
     <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="47" t="s">
+      <c r="A6" s="65" t="s">
         <v>124</v>
       </c>
-      <c r="B6" s="47"/>
-      <c r="C6" s="47"/>
-      <c r="D6" s="47"/>
-      <c r="E6" s="47"/>
-      <c r="F6" s="47"/>
+      <c r="B6" s="65"/>
+      <c r="C6" s="65"/>
+      <c r="D6" s="65"/>
+      <c r="E6" s="65"/>
+      <c r="F6" s="65"/>
       <c r="G6" s="4"/>
-      <c r="H6" s="48" t="s">
+      <c r="H6" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="I6" s="48"/>
-      <c r="J6" s="48"/>
-      <c r="K6" s="48"/>
+      <c r="I6" s="66"/>
+      <c r="J6" s="66"/>
+      <c r="K6" s="66"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="55" t="s">
+      <c r="A7" s="59" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="55"/>
-      <c r="C7" s="55"/>
-      <c r="D7" s="55"/>
-      <c r="E7" s="55"/>
-      <c r="F7" s="55"/>
+      <c r="B7" s="59"/>
+      <c r="C7" s="59"/>
+      <c r="D7" s="59"/>
+      <c r="E7" s="59"/>
+      <c r="F7" s="59"/>
       <c r="G7" s="5"/>
-      <c r="H7" s="56" t="s">
+      <c r="H7" s="60" t="s">
         <v>88</v>
       </c>
-      <c r="I7" s="56"/>
-      <c r="J7" s="56"/>
-      <c r="K7" s="56"/>
+      <c r="I7" s="60"/>
+      <c r="J7" s="60"/>
+      <c r="K7" s="60"/>
     </row>
     <row r="8" spans="1:11" s="10" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="60" t="s">
+      <c r="A8" s="47" t="s">
         <v>5</v>
       </c>
       <c r="B8" s="7" t="s">
@@ -6388,16 +6390,16 @@
       <c r="B64" s="28" t="s">
         <v>105</v>
       </c>
-      <c r="C64" s="62" t="s">
+      <c r="C64" s="49" t="s">
         <v>7</v>
       </c>
-      <c r="D64" s="62" t="s">
+      <c r="D64" s="49" t="s">
         <v>27</v>
       </c>
-      <c r="E64" s="62" t="s">
+      <c r="E64" s="49" t="s">
         <v>106</v>
       </c>
-      <c r="F64" s="62" t="s">
+      <c r="F64" s="49" t="s">
         <v>107</v>
       </c>
       <c r="G64" s="15"/>
@@ -6408,7 +6410,7 @@
     </row>
     <row r="65" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A65" s="13"/>
-      <c r="B65" s="63" t="s">
+      <c r="B65" s="50" t="s">
         <v>109</v>
       </c>
       <c r="C65" s="3">
@@ -6458,9 +6460,9 @@
       <c r="J66" s="15"/>
       <c r="K66" s="15"/>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A67" s="13"/>
-      <c r="B67" s="63" t="s">
+      <c r="B67" s="50" t="s">
         <v>110</v>
       </c>
       <c r="C67" s="3">
@@ -6647,7 +6649,7 @@
     </row>
     <row r="74" spans="1:11" s="44" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A74" s="24"/>
-      <c r="B74" s="65" t="s">
+      <c r="B74" s="52" t="s">
         <v>112</v>
       </c>
       <c r="C74" s="38"/>
@@ -6694,7 +6696,7 @@
       <c r="J76" s="22"/>
       <c r="K76" s="26"/>
     </row>
-    <row r="77" spans="1:11" ht="154.5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:11" ht="138.75" x14ac:dyDescent="0.25">
       <c r="A77" s="13">
         <v>8</v>
       </c>
@@ -6805,7 +6807,7 @@
     </row>
     <row r="82" spans="1:11" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A82" s="24"/>
-      <c r="B82" s="64" t="s">
+      <c r="B82" s="51" t="s">
         <v>118</v>
       </c>
       <c r="C82" s="26"/>
@@ -6823,7 +6825,7 @@
     </row>
     <row r="83" spans="1:11" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A83" s="24"/>
-      <c r="B83" s="64" t="s">
+      <c r="B83" s="51" t="s">
         <v>119</v>
       </c>
       <c r="C83" s="26"/>
@@ -6870,210 +6872,285 @@
       <c r="J85" s="22"/>
       <c r="K85" s="26"/>
     </row>
-    <row r="86" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:11" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A86" s="17">
         <v>9</v>
       </c>
-      <c r="B86" s="66" t="s">
-        <v>123</v>
-      </c>
-      <c r="C86" s="19">
-        <v>1</v>
-      </c>
+      <c r="B86" s="28" t="s">
+        <v>125</v>
+      </c>
+      <c r="C86" s="19"/>
       <c r="D86" s="1"/>
       <c r="E86" s="20"/>
       <c r="F86" s="20"/>
-      <c r="G86" s="21">
-        <f t="shared" ref="G86" si="10">PRODUCT(C86:F86)</f>
+      <c r="G86" s="21"/>
+      <c r="H86" s="21"/>
+      <c r="I86" s="2"/>
+      <c r="J86" s="21"/>
+      <c r="K86" s="20"/>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A87" s="13"/>
+      <c r="B87" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="C87" s="3">
         <v>1</v>
       </c>
-      <c r="H86" s="21" t="s">
-        <v>30</v>
-      </c>
-      <c r="I86" s="2">
-        <v>5000</v>
-      </c>
-      <c r="J86" s="21">
-        <f>G86*I86</f>
-        <v>5000</v>
-      </c>
-      <c r="K86" s="20"/>
-    </row>
-    <row r="87" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="24"/>
-      <c r="B87" s="25"/>
-      <c r="C87" s="26"/>
-      <c r="D87" s="27"/>
-      <c r="E87" s="27"/>
-      <c r="F87" s="27"/>
-      <c r="G87" s="27"/>
-      <c r="H87" s="26"/>
-      <c r="I87" s="26"/>
-      <c r="J87" s="22"/>
-      <c r="K87" s="26"/>
+      <c r="D87" s="3">
+        <f>D31</f>
+        <v>5.6141420298689431</v>
+      </c>
+      <c r="E87" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="F87" s="3">
+        <f>7.5/3.281</f>
+        <v>2.2858884486437061</v>
+      </c>
+      <c r="G87" s="3">
+        <f>PRODUCT(C87:F87)</f>
+        <v>1.2833302415122547</v>
+      </c>
+      <c r="H87" s="15"/>
+      <c r="I87" s="15"/>
+      <c r="J87" s="15"/>
+      <c r="K87" s="15"/>
     </row>
     <row r="88" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="17">
-        <v>10</v>
-      </c>
-      <c r="B88" s="30" t="s">
-        <v>17</v>
-      </c>
-      <c r="C88" s="19">
-        <v>1</v>
-      </c>
+      <c r="A88" s="17"/>
+      <c r="B88" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C88" s="19"/>
       <c r="D88" s="1"/>
       <c r="E88" s="20"/>
       <c r="F88" s="20"/>
-      <c r="G88" s="21">
-        <f t="shared" ref="G88" si="11">PRODUCT(C88:F88)</f>
+      <c r="G88" s="2">
+        <f>SUM(G86:G87)</f>
+        <v>1.2833302415122547</v>
+      </c>
+      <c r="H88" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="I88" s="2">
+        <v>1982.2</v>
+      </c>
+      <c r="J88" s="22">
+        <f>G88*I88</f>
+        <v>2543.8172047255912</v>
+      </c>
+      <c r="K88" s="20"/>
+    </row>
+    <row r="89" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A89" s="24"/>
+      <c r="B89" s="25"/>
+      <c r="C89" s="26"/>
+      <c r="D89" s="27"/>
+      <c r="E89" s="27"/>
+      <c r="F89" s="27"/>
+      <c r="G89" s="27"/>
+      <c r="H89" s="26"/>
+      <c r="I89" s="26"/>
+      <c r="J89" s="22"/>
+      <c r="K89" s="26"/>
+    </row>
+    <row r="90" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A90" s="17">
+        <v>10</v>
+      </c>
+      <c r="B90" s="53" t="s">
+        <v>123</v>
+      </c>
+      <c r="C90" s="19">
         <v>1</v>
       </c>
-      <c r="H88" s="21" t="s">
+      <c r="D90" s="1"/>
+      <c r="E90" s="20"/>
+      <c r="F90" s="20"/>
+      <c r="G90" s="21">
+        <f t="shared" ref="G90" si="10">PRODUCT(C90:F90)</f>
+        <v>1</v>
+      </c>
+      <c r="H90" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="I90" s="2">
+        <v>5000</v>
+      </c>
+      <c r="J90" s="21">
+        <f>G90*I90</f>
+        <v>5000</v>
+      </c>
+      <c r="K90" s="20"/>
+    </row>
+    <row r="91" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A91" s="24"/>
+      <c r="B91" s="25"/>
+      <c r="C91" s="26"/>
+      <c r="D91" s="27"/>
+      <c r="E91" s="27"/>
+      <c r="F91" s="27"/>
+      <c r="G91" s="27"/>
+      <c r="H91" s="26"/>
+      <c r="I91" s="26"/>
+      <c r="J91" s="22"/>
+      <c r="K91" s="26"/>
+    </row>
+    <row r="92" spans="1:11" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A92" s="17">
+        <v>11</v>
+      </c>
+      <c r="B92" s="30" t="s">
+        <v>17</v>
+      </c>
+      <c r="C92" s="19">
+        <v>1</v>
+      </c>
+      <c r="D92" s="1"/>
+      <c r="E92" s="20"/>
+      <c r="F92" s="20"/>
+      <c r="G92" s="21">
+        <f t="shared" ref="G92" si="11">PRODUCT(C92:F92)</f>
+        <v>1</v>
+      </c>
+      <c r="H92" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="I88" s="2">
+      <c r="I92" s="2">
         <v>500</v>
       </c>
-      <c r="J88" s="21">
-        <f>G88*I88</f>
+      <c r="J92" s="21">
+        <f>G92*I92</f>
         <v>500</v>
       </c>
-      <c r="K88" s="20"/>
-    </row>
-    <row r="89" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A89" s="17"/>
-      <c r="B89" s="31"/>
-      <c r="C89" s="19"/>
-      <c r="D89" s="1"/>
-      <c r="E89" s="20"/>
-      <c r="F89" s="20"/>
-      <c r="G89" s="2"/>
-      <c r="H89" s="21"/>
-      <c r="I89" s="2"/>
-      <c r="J89" s="22"/>
-      <c r="K89" s="20"/>
-    </row>
-    <row r="90" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A90" s="61"/>
-      <c r="B90" s="33" t="s">
+      <c r="K92" s="20"/>
+    </row>
+    <row r="93" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A93" s="17"/>
+      <c r="B93" s="31"/>
+      <c r="C93" s="19"/>
+      <c r="D93" s="1"/>
+      <c r="E93" s="20"/>
+      <c r="F93" s="20"/>
+      <c r="G93" s="2"/>
+      <c r="H93" s="21"/>
+      <c r="I93" s="2"/>
+      <c r="J93" s="22"/>
+      <c r="K93" s="20"/>
+    </row>
+    <row r="94" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A94" s="48"/>
+      <c r="B94" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="C90" s="34"/>
-      <c r="D90" s="35"/>
-      <c r="E90" s="35"/>
-      <c r="F90" s="35"/>
-      <c r="G90" s="22"/>
-      <c r="H90" s="22"/>
-      <c r="I90" s="22"/>
-      <c r="J90" s="22">
-        <f>SUM(J9:J88)</f>
-        <v>1386032.0527122186</v>
-      </c>
-      <c r="K90" s="36"/>
-    </row>
-    <row r="91" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="44"/>
-    </row>
-    <row r="92" spans="1:11" s="44" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A92" s="37"/>
-      <c r="B92" s="38" t="s">
-        <v>19</v>
-      </c>
-      <c r="C92" s="53">
-        <f>J90</f>
-        <v>1386032.0527122186</v>
-      </c>
-      <c r="D92" s="54"/>
-      <c r="E92" s="39">
-        <v>100</v>
-      </c>
-      <c r="F92" s="37"/>
-      <c r="G92" s="40"/>
-      <c r="H92" s="37"/>
-      <c r="I92" s="41"/>
-      <c r="J92" s="42"/>
-      <c r="K92" s="43"/>
-    </row>
-    <row r="93" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="44"/>
-      <c r="B93" s="38" t="s">
-        <v>21</v>
-      </c>
-      <c r="C93" s="57">
-        <v>1200000</v>
-      </c>
-      <c r="D93" s="58"/>
-      <c r="E93" s="39"/>
-    </row>
-    <row r="94" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="44"/>
-      <c r="B94" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="C94" s="57">
-        <f>C93-C96-C97</f>
-        <v>1140000</v>
-      </c>
-      <c r="D94" s="58"/>
-      <c r="E94" s="39">
-        <f>C94/C92*100</f>
-        <v>82.249180152019036</v>
-      </c>
+      <c r="C94" s="34"/>
+      <c r="D94" s="35"/>
+      <c r="E94" s="35"/>
+      <c r="F94" s="35"/>
+      <c r="G94" s="22"/>
+      <c r="H94" s="22"/>
+      <c r="I94" s="22"/>
+      <c r="J94" s="22">
+        <f>SUM(J9:J92)</f>
+        <v>1388575.8699169443</v>
+      </c>
+      <c r="K94" s="36"/>
     </row>
     <row r="95" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="44"/>
-      <c r="B95" s="38" t="s">
-        <v>26</v>
-      </c>
-      <c r="C95" s="59">
-        <f>C92-C94</f>
-        <v>246032.0527122186</v>
-      </c>
-      <c r="D95" s="59"/>
-      <c r="E95" s="39">
-        <f>100-E94</f>
-        <v>17.750819847980964</v>
-      </c>
-    </row>
-    <row r="96" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="44"/>
+    </row>
+    <row r="96" spans="1:11" s="44" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A96" s="37"/>
       <c r="B96" s="38" t="s">
-        <v>23</v>
-      </c>
-      <c r="C96" s="53">
-        <f>C93*0.03</f>
-        <v>36000</v>
-      </c>
-      <c r="D96" s="54"/>
+        <v>19</v>
+      </c>
+      <c r="C96" s="54">
+        <f>J94</f>
+        <v>1388575.8699169443</v>
+      </c>
+      <c r="D96" s="55"/>
       <c r="E96" s="39">
-        <v>3</v>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="F96" s="37"/>
+      <c r="G96" s="40"/>
+      <c r="H96" s="37"/>
+      <c r="I96" s="41"/>
+      <c r="J96" s="42"/>
+      <c r="K96" s="43"/>
     </row>
     <row r="97" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="44"/>
       <c r="B97" s="38" t="s">
+        <v>21</v>
+      </c>
+      <c r="C97" s="56">
+        <v>1200000</v>
+      </c>
+      <c r="D97" s="57"/>
+      <c r="E97" s="39"/>
+    </row>
+    <row r="98" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A98" s="44"/>
+      <c r="B98" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="C98" s="56">
+        <f>C97-C100-C101</f>
+        <v>1140000</v>
+      </c>
+      <c r="D98" s="57"/>
+      <c r="E98" s="39">
+        <f>C98/C96*100</f>
+        <v>82.098502840049164</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A99" s="44"/>
+      <c r="B99" s="38" t="s">
+        <v>26</v>
+      </c>
+      <c r="C99" s="58">
+        <f>C96-C98</f>
+        <v>248575.8699169443</v>
+      </c>
+      <c r="D99" s="58"/>
+      <c r="E99" s="39">
+        <f>100-E98</f>
+        <v>17.901497159950836</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A100" s="44"/>
+      <c r="B100" s="38" t="s">
+        <v>23</v>
+      </c>
+      <c r="C100" s="54">
+        <f>C97*0.03</f>
+        <v>36000</v>
+      </c>
+      <c r="D100" s="55"/>
+      <c r="E100" s="39">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A101" s="44"/>
+      <c r="B101" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="C97" s="53">
-        <f>C93*0.02</f>
+      <c r="C101" s="54">
+        <f>C97*0.02</f>
         <v>24000</v>
       </c>
-      <c r="D97" s="54"/>
-      <c r="E97" s="39">
+      <c r="D101" s="55"/>
+      <c r="E101" s="39">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="C96:D96"/>
-    <mergeCell ref="C97:D97"/>
-    <mergeCell ref="A7:F7"/>
-    <mergeCell ref="H7:K7"/>
-    <mergeCell ref="C92:D92"/>
-    <mergeCell ref="C93:D93"/>
-    <mergeCell ref="C94:D94"/>
-    <mergeCell ref="C95:D95"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="H6:K6"/>
     <mergeCell ref="A1:K1"/>
@@ -7081,6 +7158,14 @@
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A5:K5"/>
+    <mergeCell ref="C100:D100"/>
+    <mergeCell ref="C101:D101"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="H7:K7"/>
+    <mergeCell ref="C96:D96"/>
+    <mergeCell ref="C97:D97"/>
+    <mergeCell ref="C98:D98"/>
+    <mergeCell ref="C99:D99"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="80" orientation="portrait" r:id="rId1"/>

</xml_diff>